<commit_message>
Real Another Day Coffee menu, EN/VI, cart + WhatsApp ordering
- Replace sample data with the real bilingual menu (27 items) and rename the
  café to Another Day Coffee; real address, hours (07:00–18:00) and Maps link
- Add EN/VI language selector (auto-detects Vietnamese phones, persisted);
  bilingual UI strings, About/Contacts copy, categories and item names
- Add cart: add/stepper on cards, floating order bar, bottom-sheet with table
  number + note, sends the order to the manager's WhatsApp (CAFE.whatsapp)
- Add logo support (CAFE.logo) in header + drawer
- Tighten margins/spacing and tone down the koi so it stays non-distracting
- Bilingual data pipeline: build_menu.py + import/export handle name_vi /
  category_vi (description now optional)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/menu.xlsx
+++ b/backend/menu.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,31 +413,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>category_vi</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>name_vi</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
         <is>
           <t>price</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -461,22 +459,28 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Breakfast</t>
+          <t>Vietnamese Coffee</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Avocado Toast</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>75000</v>
+          <t>Cà phê Việt</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Black Coffee</t>
+        </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Sourdough, smashed avocado, chili flakes</t>
-        </is>
-      </c>
+          <t>Cafe đen</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>20000</v>
+      </c>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -484,22 +488,28 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Breakfast</t>
+          <t>Vietnamese Coffee</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Greek Yogurt Bowl</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>60000</v>
+          <t>Cà phê Việt</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Condensed Milk Coffee</t>
+        </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Yogurt, granola, honey, seasonal fruit</t>
-        </is>
-      </c>
+          <t>Cafe sữa</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>25000</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -507,22 +517,28 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Sandwiches</t>
+          <t>Vietnamese Coffee</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Turkey Club</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>95000</v>
+          <t>Cà phê Việt</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Sai Gon Condensed Milk Coffee</t>
+        </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Turkey, bacon, lettuce, tomato on ciabatta</t>
-        </is>
-      </c>
+          <t>Cafe sữa đá Sài Gòn</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>30000</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -530,22 +546,28 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Sandwiches</t>
+          <t>Vietnamese Coffee</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Caprese Panini</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>85000</v>
+          <t>Cà phê Việt</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Salt Coffee</t>
+        </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Mozzarella, tomato, basil, balsamic glaze</t>
-        </is>
-      </c>
+          <t>Cafe muối</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>35000</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -553,22 +575,28 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Salads</t>
+          <t>Vietnamese Coffee</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Caesar Salad</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>80000</v>
+          <t>Cà phê Việt</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>White Coffee</t>
+        </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Romaine, parmesan, croutons, Caesar dressing</t>
-        </is>
-      </c>
+          <t>Bạc xỉu</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>30000</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -576,22 +604,28 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Salads</t>
+          <t>Vietnamese Coffee</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Quinoa Power Bowl</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>98000</v>
+          <t>Cà phê Việt</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Salt White Coffee</t>
+        </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Quinoa, chickpeas, kale, lemon tahini</t>
-        </is>
-      </c>
+          <t>Bạc xỉu kem muối</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>35000</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -599,22 +633,28 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Drinks</t>
+          <t>Italian Coffee</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Iced Latte</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
+          <t>Cà phê Ý</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Espresso</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Espresso</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
         <v>45000</v>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Double espresso over ice with milk</t>
-        </is>
-      </c>
+      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -622,22 +662,28 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Drinks</t>
+          <t>Italian Coffee</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Fresh Lemonade</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>35000</v>
+          <t>Cà phê Ý</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Americano</t>
+        </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>House-made, lightly sweetened</t>
-        </is>
-      </c>
+          <t>Americano</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>45000</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -645,22 +691,28 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Desserts</t>
+          <t>Italian Coffee</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Chocolate Brownie</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>38000</v>
+          <t>Cà phê Ý</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Cappuccino</t>
+        </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Fudgy, walnuts, sea salt</t>
-        </is>
-      </c>
+          <t>Cappuccino</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -668,22 +720,521 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Desserts</t>
+          <t>Italian Coffee</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fruit Tart</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
+          <t>Cà phê Ý</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Latte</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Latte</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Italian Coffee</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Cà phê Ý</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Flat White</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Flat White</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Coldbrew</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Coldbrew</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Coldbrew Original</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Truyền thống</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>40000</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Coldbrew</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Coldbrew</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Sunshine</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Nắng</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
         <v>45000</v>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Pastry cream, glazed seasonal fruit</t>
-        </is>
-      </c>
+      <c r="G14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Coldbrew</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Coldbrew</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Lemon Coldbrew</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Coldbrew chanh</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>40000</v>
+      </c>
+      <c r="G15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Coldbrew</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Coldbrew</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Orange Coldbrew</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Coldbrew cam</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>40000</v>
+      </c>
+      <c r="G16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Refreshing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Giải khát</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Pomegranate Tea</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Trà lựu</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>35000</v>
+      </c>
+      <c r="G17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Refreshing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Giải khát</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Longan Tea</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Trà long nhãn</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>35000</v>
+      </c>
+      <c r="G18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Refreshing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Giải khát</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Hibiscus Tea</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Trà atiso</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>35000</v>
+      </c>
+      <c r="G19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Refreshing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Giải khát</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Orange Cinnamon Honey Tea</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Trà cam quế mật ong</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>35000</v>
+      </c>
+      <c r="G20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Khác</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Hibiscus Lemon</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Chanh atiso</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>30000</v>
+      </c>
+      <c r="G21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Khác</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Orange Juice</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Cam</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>30000</v>
+      </c>
+      <c r="G22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Khác</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Choco Latte</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Choco latte</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>30000</v>
+      </c>
+      <c r="G23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Khác</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Salt Chocolate</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Choco latte kem muối</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>35000</v>
+      </c>
+      <c r="G24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Khác</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Iced Lemon Yogurt</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Yogurt đá chanh</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>30000</v>
+      </c>
+      <c r="G25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Khác</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Peach Yogurt</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Yogurt đào</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>35000</v>
+      </c>
+      <c r="G26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Soft Drink</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Nước ngọt</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Nước suối</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>10000</v>
+      </c>
+      <c r="G27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Soft Drink</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Nước ngọt</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Coca Light</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Coca Light</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>20000</v>
+      </c>
+      <c r="G28" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>